<commit_message>
updating market tracker, schedular, and excel
Former-commit-id: b70f752634a6505d8286f7f28c55553c8f31ffbe
</commit_message>
<xml_diff>
--- a/assets/PredictionMarkets/Prediction_Market_Master.xlsx
+++ b/assets/PredictionMarkets/Prediction_Market_Master.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Website\connorbuttonweb.github.io\assets\PredictionMarkets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11F2F0A0-E2D0-43DE-BD2D-243500615301}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56DE9076-53D3-49AE-AFBE-BA2324931265}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,24 +19,15 @@
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -47,7 +38,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -55,30 +46,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -381,21 +354,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A1" s="1"/>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-    </row>
-  </sheetData>
+  <sheetData/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>